<commit_message>
Added lookups for filing requirement codes
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tpoongundranar\Documents\Urban\NCCS\nccs-data-bmf\data\lookup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675A64CC-3CDB-4B6A-BC34-02DEE7F5FDD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A261B831-7AC8-4A55-A3D2-CBC26664A0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
   </bookViews>
   <sheets>
     <sheet name="status_code" sheetId="1" r:id="rId1"/>
     <sheet name="asset_code" sheetId="2" r:id="rId2"/>
-    <sheet name="income_code" sheetId="3" r:id="rId3"/>
+    <sheet name="filing_requirement_code" sheetId="4" r:id="rId3"/>
+    <sheet name="income_code" sheetId="3" r:id="rId4"/>
+    <sheet name="pf_filing_requirement_code" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="43">
   <si>
     <t>status_code</t>
   </si>
@@ -101,6 +103,72 @@
   </si>
   <si>
     <t>income_code_effective_date</t>
+  </si>
+  <si>
+    <t>filing_requirement_code</t>
+  </si>
+  <si>
+    <t>filing_requirement_code_definition</t>
+  </si>
+  <si>
+    <t>filing_requirement_code_effective_date</t>
+  </si>
+  <si>
+    <t>990 - Not required to file (all other)</t>
+  </si>
+  <si>
+    <t>990 (all other) or 990EZ return</t>
+  </si>
+  <si>
+    <t>990 - Required to file Form 990-N - Income less than $50,000 per year</t>
+  </si>
+  <si>
+    <t>990 - Group return</t>
+  </si>
+  <si>
+    <t>990 - Required to file Form 990-BL, Black Lung Trusts</t>
+  </si>
+  <si>
+    <t>990 - Not required to file (church)</t>
+  </si>
+  <si>
+    <t>990 - Government 501(c)(1)</t>
+  </si>
+  <si>
+    <t>990 - Not required to file (religious organization)</t>
+  </si>
+  <si>
+    <t>990 - Not required to file (instrumentalities of states or political subdivisions)</t>
+  </si>
+  <si>
+    <t>pf_filing_requirement_code</t>
+  </si>
+  <si>
+    <t>pf_filing_requirement_code_definition</t>
+  </si>
+  <si>
+    <t>pf_filing_requirement_code_description</t>
+  </si>
+  <si>
+    <t>pf_filing_requirement_code_effective_date</t>
+  </si>
+  <si>
+    <t>No 990-PF return</t>
+  </si>
+  <si>
+    <t>990-PF return</t>
+  </si>
+  <si>
+    <t>Return due 5 months or the 15th day of the 5th month after the end of the taxable year.</t>
+  </si>
+  <si>
+    <t>Revoked, required to file Form 990-PF and Form 1120.</t>
+  </si>
+  <si>
+    <t>Presumptive</t>
+  </si>
+  <si>
+    <t>No return due</t>
   </si>
 </sst>
 </file>
@@ -656,6 +724,126 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8C9601-88C1-4ACF-A4DB-1D9ED72BCB8C}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10">
+        <v>20241213</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0CDB35C-585B-4DD3-B01E-2ED46C16F7EF}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -784,4 +972,84 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F0813D5-4CF6-451E-8856-3E71508FC2CF}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5">
+        <v>20241213</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add parent organization lookup
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tpoongundranar\Documents\Urban\NCCS\nccs-data-bmf\data\lookup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F943B9F7-A4D6-4DBE-A5B7-AB3636CD145D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6569F1-4400-4902-AD61-11DF37067A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="5" activeTab="5" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
   </bookViews>
   <sheets>
     <sheet name="status_code" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="ntee_code" sheetId="6" r:id="rId6"/>
     <sheet name="ntee_code_activity_type" sheetId="7" r:id="rId7"/>
     <sheet name="ntee_code_major_group" sheetId="8" r:id="rId8"/>
+    <sheet name="parent_organization" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="1238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="1552">
   <si>
     <t>status_code</t>
   </si>
@@ -3757,6 +3758,948 @@
   </si>
   <si>
     <t>UNDEFINED</t>
+  </si>
+  <si>
+    <t>Air Line Dispatchers Association</t>
+  </si>
+  <si>
+    <t>ADA</t>
+  </si>
+  <si>
+    <t>Air Line Pilots Association; International</t>
+  </si>
+  <si>
+    <t>APA</t>
+  </si>
+  <si>
+    <t>Allied and Technical Workers District 50 International Union</t>
+  </si>
+  <si>
+    <t>ATW-50</t>
+  </si>
+  <si>
+    <t>Allied Industrial Workers of America International Union</t>
+  </si>
+  <si>
+    <t>AIWA</t>
+  </si>
+  <si>
+    <t>Aluminum Workers International Union</t>
+  </si>
+  <si>
+    <t>AWU</t>
+  </si>
+  <si>
+    <t>Amalgamated clothing Workers of America</t>
+  </si>
+  <si>
+    <t>ACW</t>
+  </si>
+  <si>
+    <t>Amalgamated Meat cutters &amp; Butcher Workmen of North America</t>
+  </si>
+  <si>
+    <t>MCBW</t>
+  </si>
+  <si>
+    <t>Amalgamated Transit Unit (F/K/A SERE)</t>
+  </si>
+  <si>
+    <t>ATU</t>
+  </si>
+  <si>
+    <t>Amalgamated Transit Union Women’s International Auxiliary</t>
+  </si>
+  <si>
+    <t>ATU-Aux</t>
+  </si>
+  <si>
+    <t>American Communications Association (Ind.)</t>
+  </si>
+  <si>
+    <t>ACA</t>
+  </si>
+  <si>
+    <t>American Federation of Government Employees</t>
+  </si>
+  <si>
+    <t>AFGE</t>
+  </si>
+  <si>
+    <t>American Federation of Grain Millers</t>
+  </si>
+  <si>
+    <t>AFGM</t>
+  </si>
+  <si>
+    <t>American Federation of Labor and Congress of Industrial Organizations</t>
+  </si>
+  <si>
+    <t>AFL-CIO</t>
+  </si>
+  <si>
+    <t>American Federation of Labor and Congress of Industrial Organizations — Auxiliaries</t>
+  </si>
+  <si>
+    <t>AFL-CIO Aux</t>
+  </si>
+  <si>
+    <t>American Federation of Musicians of the U.S. and Canada</t>
+  </si>
+  <si>
+    <t>AFM</t>
+  </si>
+  <si>
+    <t>American Federation of State, County and Municipal Employees</t>
+  </si>
+  <si>
+    <t>SCME</t>
+  </si>
+  <si>
+    <t>American Federation of Teachers</t>
+  </si>
+  <si>
+    <t>AFT</t>
+  </si>
+  <si>
+    <t>American Federation of Technical Engineers</t>
+  </si>
+  <si>
+    <t>FTE</t>
+  </si>
+  <si>
+    <t>American Flint Glass Workers Union of North American</t>
+  </si>
+  <si>
+    <t>FGWU</t>
+  </si>
+  <si>
+    <t>American Newspaper Guild</t>
+  </si>
+  <si>
+    <t>ANG</t>
+  </si>
+  <si>
+    <t>American Railway Supervisors</t>
+  </si>
+  <si>
+    <t>ARS</t>
+  </si>
+  <si>
+    <t>Bakery and Confectionery Workers’ International Union of America</t>
+  </si>
+  <si>
+    <t>BCWI</t>
+  </si>
+  <si>
+    <t>Bill Posters, Billers and Distributors of the U.S. and Canada International Alliance</t>
+  </si>
+  <si>
+    <t>BPBD</t>
+  </si>
+  <si>
+    <t>Boot &amp; Shoe Workers Union</t>
+  </si>
+  <si>
+    <t>BSWU</t>
+  </si>
+  <si>
+    <t>Bricklayers, Masons and Plasterers’ International Union of America</t>
+  </si>
+  <si>
+    <t>BMPI</t>
+  </si>
+  <si>
+    <t>Brotherhood of Locomotive Engineers</t>
+  </si>
+  <si>
+    <t>BLE</t>
+  </si>
+  <si>
+    <t>Brotherhood of Locomotive Engineers Auxiliary</t>
+  </si>
+  <si>
+    <t>BLE-Aux</t>
+  </si>
+  <si>
+    <t>Brotherhood of Maintenance of Way Employees</t>
+  </si>
+  <si>
+    <t>BMWE</t>
+  </si>
+  <si>
+    <t>Brotherhood of Maintenance of Way Employees Ladies Auxiliaries</t>
+  </si>
+  <si>
+    <t>BMWE-Aux</t>
+  </si>
+  <si>
+    <t>Brotherhood of Railroad Signalmen</t>
+  </si>
+  <si>
+    <t>BRS</t>
+  </si>
+  <si>
+    <t>Brotherhood of Railway, Airline and Steamship Clerks, Freight Handlers</t>
+  </si>
+  <si>
+    <t>BRAC</t>
+  </si>
+  <si>
+    <t>Brotherhood of Railway Carmen of America</t>
+  </si>
+  <si>
+    <t>RCA</t>
+  </si>
+  <si>
+    <t>Brotherhood of Shoe and Allied Craftsmen</t>
+  </si>
+  <si>
+    <t>NSAC</t>
+  </si>
+  <si>
+    <t>Brotherhood of Sleeping Car Porters, Train Chair Car Coach Porters &amp; Attend.</t>
+  </si>
+  <si>
+    <t>SCP</t>
+  </si>
+  <si>
+    <t>Brotherhood of Utility Workers of New England</t>
+  </si>
+  <si>
+    <t>UWNE</t>
+  </si>
+  <si>
+    <t>Christian Labor Association of the United States of America (Ind.)</t>
+  </si>
+  <si>
+    <t>CLA</t>
+  </si>
+  <si>
+    <t>Cigar Maker’s International Union of America</t>
+  </si>
+  <si>
+    <t>CIUA</t>
+  </si>
+  <si>
+    <t>Communication Workers of America</t>
+  </si>
+  <si>
+    <t>CWA</t>
+  </si>
+  <si>
+    <t>Cooper’s International Union of North America</t>
+  </si>
+  <si>
+    <t>CIU</t>
+  </si>
+  <si>
+    <t>Cordova District Fisheries Union</t>
+  </si>
+  <si>
+    <t>CDFU</t>
+  </si>
+  <si>
+    <t>Distillery, Rectifying, Wine and Allied Workers International Union</t>
+  </si>
+  <si>
+    <t>DWAW</t>
+  </si>
+  <si>
+    <t>Flight Engineers’ International Association</t>
+  </si>
+  <si>
+    <t>FEIA</t>
+  </si>
+  <si>
+    <t>Glass Bottle Blowers Association of the U.S. and Canada</t>
+  </si>
+  <si>
+    <t>GBBA</t>
+  </si>
+  <si>
+    <t>Granite Cutter’s International Association of America</t>
+  </si>
+  <si>
+    <t>GCIA</t>
+  </si>
+  <si>
+    <t>Hotel and Restaurant Employees’ and Bartenders International Union</t>
+  </si>
+  <si>
+    <t>HREU</t>
+  </si>
+  <si>
+    <t>Independent Watchmen’s Association</t>
+  </si>
+  <si>
+    <t>WA</t>
+  </si>
+  <si>
+    <t>Insurance Workers International Union</t>
+  </si>
+  <si>
+    <t>IWIU</t>
+  </si>
+  <si>
+    <t>International Alliance of Theatrical State Employees &amp; Moving Picture Operators</t>
+  </si>
+  <si>
+    <t>LATSE</t>
+  </si>
+  <si>
+    <t>International Association of Fire Fighters</t>
+  </si>
+  <si>
+    <t>LAFF</t>
+  </si>
+  <si>
+    <t>International Association of Fire Fighters Auxiliary</t>
+  </si>
+  <si>
+    <t>LAFF-Aux</t>
+  </si>
+  <si>
+    <t>International Association of Heat and Frost Insulators &amp; Asbestos Workers</t>
+  </si>
+  <si>
+    <t>AWIA</t>
+  </si>
+  <si>
+    <t>International Association of Machinists &amp; Aerospace Workers</t>
+  </si>
+  <si>
+    <t>LAM</t>
+  </si>
+  <si>
+    <t>International Association of Marble, Slate &amp; Stone Polishers, etc.</t>
+  </si>
+  <si>
+    <t>MSSP</t>
+  </si>
+  <si>
+    <t>International Brotherhood of Boilermakers, Iron Ship Builders, Blacksmiths</t>
+  </si>
+  <si>
+    <t>BMIS</t>
+  </si>
+  <si>
+    <t>International Brotherhood of Electrical Workers</t>
+  </si>
+  <si>
+    <t>IBEW</t>
+  </si>
+  <si>
+    <t>International Brotherhood of Firemen and Oilers</t>
+  </si>
+  <si>
+    <t>FOIB</t>
+  </si>
+  <si>
+    <t>International Brotherhood of Painters and Allied Trades</t>
+  </si>
+  <si>
+    <t>BPAT</t>
+  </si>
+  <si>
+    <t>International Brotherhood of Potters and Allied Workers</t>
+  </si>
+  <si>
+    <t>BOP</t>
+  </si>
+  <si>
+    <t>International Brotherhood of Teamsters, Chauffeurs, Warehousemen &amp; Helpers of America (Ind.)</t>
+  </si>
+  <si>
+    <t>TCWH</t>
+  </si>
+  <si>
+    <t>International Chemical Workers Union</t>
+  </si>
+  <si>
+    <t>ICWU</t>
+  </si>
+  <si>
+    <t>International Die Sinker’s Conference</t>
+  </si>
+  <si>
+    <t>DSC</t>
+  </si>
+  <si>
+    <t>International Guards Union of America</t>
+  </si>
+  <si>
+    <t>GUA</t>
+  </si>
+  <si>
+    <t>International Jewelry Workers Union</t>
+  </si>
+  <si>
+    <t>IJWU</t>
+  </si>
+  <si>
+    <t>International Ladies Garment Workers Union</t>
+  </si>
+  <si>
+    <t>ILGW</t>
+  </si>
+  <si>
+    <t>International Leather Goods, Plastic &amp; Novelty Workers Union</t>
+  </si>
+  <si>
+    <t>LGPW</t>
+  </si>
+  <si>
+    <t>International Longshoremen’s and Warehousemen’s Union</t>
+  </si>
+  <si>
+    <t>ILWU</t>
+  </si>
+  <si>
+    <t>International Longshoremens Association (Ind.)</t>
+  </si>
+  <si>
+    <t>ILA</t>
+  </si>
+  <si>
+    <t>International McClass Sailboat Racing Association (Ind.)</t>
+  </si>
+  <si>
+    <t>IMCCSRA</t>
+  </si>
+  <si>
+    <t>International Mailers Union</t>
+  </si>
+  <si>
+    <t>IMU</t>
+  </si>
+  <si>
+    <t>International Molders &amp; Allied Workers Union</t>
+  </si>
+  <si>
+    <t>MAWU</t>
+  </si>
+  <si>
+    <t>International Organization of Masters, Mates &amp; Pilots</t>
+  </si>
+  <si>
+    <t>MMPI</t>
+  </si>
+  <si>
+    <t>International Plate Printers, Die Stampers &amp; Engravers Union of North America</t>
+  </si>
+  <si>
+    <t>PPEU</t>
+  </si>
+  <si>
+    <t>International Printing Pressmen &amp; Assistants Union of North America</t>
+  </si>
+  <si>
+    <t>IPP</t>
+  </si>
+  <si>
+    <t>International Stereotypers &amp; Electrotypes Union of North America</t>
+  </si>
+  <si>
+    <t>ISEU</t>
+  </si>
+  <si>
+    <t>International Typographical Union of North America</t>
+  </si>
+  <si>
+    <t>ITU</t>
+  </si>
+  <si>
+    <t>International Union of Electrical Radio and Machine Workers</t>
+  </si>
+  <si>
+    <t>IUE</t>
+  </si>
+  <si>
+    <t>International Union of Elevator Constructors</t>
+  </si>
+  <si>
+    <t>ECI</t>
+  </si>
+  <si>
+    <t>International Union of Journeymen Horseshoers of the U.S. and Canada</t>
+  </si>
+  <si>
+    <t>HSIU</t>
+  </si>
+  <si>
+    <t>International Union of Life Insurance Agents</t>
+  </si>
+  <si>
+    <t>LIA</t>
+  </si>
+  <si>
+    <t>International Union of United Brewery, Flour Cereal, Soft Drinks and Distillery Workers of America</t>
+  </si>
+  <si>
+    <t>BSDW</t>
+  </si>
+  <si>
+    <t>International Woodworkers of America</t>
+  </si>
+  <si>
+    <t>IWA</t>
+  </si>
+  <si>
+    <t>Journeymen Barbers, Hairdressers, Cosmetologists &amp; Proprietors A/K/A Barbers, Beauticians &amp; Allied Industries</t>
+  </si>
+  <si>
+    <t>BHCI/BBAI</t>
+  </si>
+  <si>
+    <t>Laborers International Union of North America</t>
+  </si>
+  <si>
+    <t>HCL</t>
+  </si>
+  <si>
+    <t>Laundry &amp; Dry Cleaning Workers International Union</t>
+  </si>
+  <si>
+    <t>LDCI</t>
+  </si>
+  <si>
+    <t>Laundry &amp; Dry Cleaning Workers International Union (Ind.)</t>
+  </si>
+  <si>
+    <t>LWIU</t>
+  </si>
+  <si>
+    <t>Leather Workers International Union of America</t>
+  </si>
+  <si>
+    <t>LWIUA</t>
+  </si>
+  <si>
+    <t>Marine &amp; Shipbuilding Workers of America, Industrial Union</t>
+  </si>
+  <si>
+    <t>MSWA</t>
+  </si>
+  <si>
+    <t>Metal Polishers, Buffers, Platers &amp; Helpers International Union</t>
+  </si>
+  <si>
+    <t>MPBP</t>
+  </si>
+  <si>
+    <t>National Alliance of Postal &amp; Federal Employees (F/K/A NAPE)</t>
+  </si>
+  <si>
+    <t>NAPFE</t>
+  </si>
+  <si>
+    <t>National Association of Broadcast Employees &amp; Technicians</t>
+  </si>
+  <si>
+    <t>NABET</t>
+  </si>
+  <si>
+    <t>National Association of Government Employees (Ind.)</t>
+  </si>
+  <si>
+    <t>NAGE</t>
+  </si>
+  <si>
+    <t>National Association of Letter Carriers of the U.S.A.</t>
+  </si>
+  <si>
+    <t>NALC</t>
+  </si>
+  <si>
+    <t>National Association of Post Office Mail Handlers, Messengers and Group Leaders</t>
+  </si>
+  <si>
+    <t>POMH</t>
+  </si>
+  <si>
+    <t>National Congress of Industrial Waterproofing &amp; Misc. Workers of America (Ind.)</t>
+  </si>
+  <si>
+    <t>NCIWMWA</t>
+  </si>
+  <si>
+    <t>National Federation of Federal Employees (Ind.)</t>
+  </si>
+  <si>
+    <t>NFFE</t>
+  </si>
+  <si>
+    <t>National League of Postmasters of the U.S. (Ind.)</t>
+  </si>
+  <si>
+    <t>NLP</t>
+  </si>
+  <si>
+    <t>National Marine Engineers Beneficial Assn. Of the U.S.A.</t>
+  </si>
+  <si>
+    <t>MEBA</t>
+  </si>
+  <si>
+    <t>National Rural Letter Carriers’ Association (Ind.)</t>
+  </si>
+  <si>
+    <t>RLCA</t>
+  </si>
+  <si>
+    <t>National Treasury Employees Union (F/K/A NAIRE) (Ind.)</t>
+  </si>
+  <si>
+    <t>NTEU</t>
+  </si>
+  <si>
+    <t>Office &amp; Professional Employees International Union</t>
+  </si>
+  <si>
+    <t>OEIU</t>
+  </si>
+  <si>
+    <t>Oil, Chemical &amp; Atomic Workers International Union</t>
+  </si>
+  <si>
+    <t>OCAW</t>
+  </si>
+  <si>
+    <t>Operative Plasterer’s &amp; Cement Masons International Association</t>
+  </si>
+  <si>
+    <t>PCM</t>
+  </si>
+  <si>
+    <t>Pattern Makers’ League of North America</t>
+  </si>
+  <si>
+    <t>PML</t>
+  </si>
+  <si>
+    <t>Railroad Yardmasters of America</t>
+  </si>
+  <si>
+    <t>RYA</t>
+  </si>
+  <si>
+    <t>Railway Patrolmen’s International Union</t>
+  </si>
+  <si>
+    <t>IURP</t>
+  </si>
+  <si>
+    <t>Retail Clerks International Association</t>
+  </si>
+  <si>
+    <t>RCIA</t>
+  </si>
+  <si>
+    <t>Retail, Wholesale &amp; Department Store Union</t>
+  </si>
+  <si>
+    <t>RWDS</t>
+  </si>
+  <si>
+    <t>Seafarers’ International Union of North America</t>
+  </si>
+  <si>
+    <t>SIU</t>
+  </si>
+  <si>
+    <t>Service Employees International Union (F/K/A DSE)</t>
+  </si>
+  <si>
+    <t>SEIU</t>
+  </si>
+  <si>
+    <t>Sheet Metal Workers International Association</t>
+  </si>
+  <si>
+    <t>SMW</t>
+  </si>
+  <si>
+    <t>Stove, Furnace &amp; Allied Appliance Workers International Union of North America</t>
+  </si>
+  <si>
+    <t>SFAW</t>
+  </si>
+  <si>
+    <t>Textile Workers Union of America</t>
+  </si>
+  <si>
+    <t>TWUA</t>
+  </si>
+  <si>
+    <t>Tobacco Workers International Union</t>
+  </si>
+  <si>
+    <t>TWIU</t>
+  </si>
+  <si>
+    <t>Transport Workers Union of America</t>
+  </si>
+  <si>
+    <t>TWU</t>
+  </si>
+  <si>
+    <t>United Association of Journeymen &amp; Apprentices of the Plumbing &amp; Pipe Fitting Industry</t>
+  </si>
+  <si>
+    <t>PPF</t>
+  </si>
+  <si>
+    <t>United Automobile, Aerospace &amp; Agricultural Workers of America</t>
+  </si>
+  <si>
+    <t>UAW</t>
+  </si>
+  <si>
+    <t>United Brick &amp; Clay Workers of America</t>
+  </si>
+  <si>
+    <t>BCW</t>
+  </si>
+  <si>
+    <t>United Brotherhood of Carpenters &amp; Joiners of America</t>
+  </si>
+  <si>
+    <t>BCJ</t>
+  </si>
+  <si>
+    <t>United Cement, Lime &amp; Gypsum Workers International Union</t>
+  </si>
+  <si>
+    <t>CLGW</t>
+  </si>
+  <si>
+    <t>United Electrical, Radio &amp; Machine Workers of Americ (Ind.)</t>
+  </si>
+  <si>
+    <t>UE</t>
+  </si>
+  <si>
+    <t>United Furniture Workers of America</t>
+  </si>
+  <si>
+    <t>FWA</t>
+  </si>
+  <si>
+    <t>United Garment Workers of America</t>
+  </si>
+  <si>
+    <t>UGWA</t>
+  </si>
+  <si>
+    <t>United Glass &amp; Ceramic Workers of North America</t>
+  </si>
+  <si>
+    <t>GCW</t>
+  </si>
+  <si>
+    <t>United Hatters Cap &amp; Military Workers International Union</t>
+  </si>
+  <si>
+    <t>HCMW</t>
+  </si>
+  <si>
+    <t>United Mine Workers of America (Ind.)</t>
+  </si>
+  <si>
+    <t>UMW</t>
+  </si>
+  <si>
+    <t>United Paperworkers International Union (from the merger of PMPW &amp; PSPM)</t>
+  </si>
+  <si>
+    <t>UPIU</t>
+  </si>
+  <si>
+    <t>United Plant Guard Workers of America (Ind.)</t>
+  </si>
+  <si>
+    <t>PGW</t>
+  </si>
+  <si>
+    <t>United Rubber, Cork, Linoleum &amp; Plastic Workers of America</t>
+  </si>
+  <si>
+    <t>RWA</t>
+  </si>
+  <si>
+    <t>United Shoe Workers of America</t>
+  </si>
+  <si>
+    <t>SWA</t>
+  </si>
+  <si>
+    <t>United Slate, Tile &amp; Composition Roofers, Damp &amp; Waterproof Workers of Assn.</t>
+  </si>
+  <si>
+    <t>RDWA</t>
+  </si>
+  <si>
+    <t>United Steelworkers of America</t>
+  </si>
+  <si>
+    <t>USW</t>
+  </si>
+  <si>
+    <t>United Telegraph Workers</t>
+  </si>
+  <si>
+    <t>UTW</t>
+  </si>
+  <si>
+    <t>United Textile Workers of America</t>
+  </si>
+  <si>
+    <t>UTWA</t>
+  </si>
+  <si>
+    <t>United Transport Service Employees of American International Union</t>
+  </si>
+  <si>
+    <t>TSEA</t>
+  </si>
+  <si>
+    <t>United Transportation Union</t>
+  </si>
+  <si>
+    <t>UTU</t>
+  </si>
+  <si>
+    <t>Upholsterers’ International Union of N.A.</t>
+  </si>
+  <si>
+    <t>UIUA</t>
+  </si>
+  <si>
+    <t>Utilities Workers Union of America</t>
+  </si>
+  <si>
+    <t>UWUA</t>
+  </si>
+  <si>
+    <t>Window Glass Cutters League of America</t>
+  </si>
+  <si>
+    <t>GCLA</t>
+  </si>
+  <si>
+    <t>Wood, Wine &amp; Metal Lathers’ International Union</t>
+  </si>
+  <si>
+    <t>IUWM</t>
+  </si>
+  <si>
+    <t>American Association of University Women</t>
+  </si>
+  <si>
+    <t>AWARE</t>
+  </si>
+  <si>
+    <t>American Medical Association</t>
+  </si>
+  <si>
+    <t>AMA</t>
+  </si>
+  <si>
+    <t>American Veterans of World War II</t>
+  </si>
+  <si>
+    <t>AM VETS</t>
+  </si>
+  <si>
+    <t>Benevolent and Protective Order of Elks</t>
+  </si>
+  <si>
+    <t>BP OE</t>
+  </si>
+  <si>
+    <t>BSA</t>
+  </si>
+  <si>
+    <t>Camp Fire Girls</t>
+  </si>
+  <si>
+    <t>CFC</t>
+  </si>
+  <si>
+    <t>Daughters of the American Revolution</t>
+  </si>
+  <si>
+    <t>DAR</t>
+  </si>
+  <si>
+    <t>Disabled American Veterans</t>
+  </si>
+  <si>
+    <t>DAD</t>
+  </si>
+  <si>
+    <t>Future Farmers of America</t>
+  </si>
+  <si>
+    <t>FF A</t>
+  </si>
+  <si>
+    <t>Girl Scouts of America</t>
+  </si>
+  <si>
+    <t>GSA</t>
+  </si>
+  <si>
+    <t>Knights of Columbus</t>
+  </si>
+  <si>
+    <t>KC</t>
+  </si>
+  <si>
+    <t>National Association for the Advancement of Colored People</t>
+  </si>
+  <si>
+    <t>NAACP</t>
+  </si>
+  <si>
+    <t>Parents Teachers Association</t>
+  </si>
+  <si>
+    <t>Society for the Preservation and Encouragement of Barbershop Quartet Singing of America</t>
+  </si>
+  <si>
+    <t>SPOUSED</t>
+  </si>
+  <si>
+    <t>Veterans of Foreign Wars</t>
+  </si>
+  <si>
+    <t>VFW</t>
+  </si>
+  <si>
+    <t>Young Men’s Christian Association</t>
+  </si>
+  <si>
+    <t>YMCA</t>
+  </si>
+  <si>
+    <t>Young Women’s Christian Association</t>
+  </si>
+  <si>
+    <t>YWCA</t>
+  </si>
+  <si>
+    <t>parent_org_name</t>
+  </si>
+  <si>
+    <t>abbreviation</t>
+  </si>
+  <si>
+    <t>gen</t>
+  </si>
+  <si>
+    <t>PTA</t>
   </si>
 </sst>
 </file>
@@ -3766,8 +4709,16 @@
   <numFmts count="1">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -3783,7 +4734,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -3791,14 +4742,81 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14084,4 +15102,1724 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C13D203-B39D-4F56-8E03-8D481588AEBE}">
+  <dimension ref="A1:C157"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>1548</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>1239</v>
+      </c>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C3" s="7"/>
+    </row>
+    <row r="4" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>1243</v>
+      </c>
+      <c r="C4" s="7">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C5" s="7">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>1247</v>
+      </c>
+      <c r="C6" s="7">
+        <v>1403</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1249</v>
+      </c>
+      <c r="C7" s="7">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C8" s="7">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C9" s="7">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>1254</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C10" s="7">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C11" s="7">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>1258</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C12" s="7">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C13" s="7">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>1264</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C15" s="7">
+        <v>1417</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>1266</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C16" s="7">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C17" s="7">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C18" s="7">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>1273</v>
+      </c>
+      <c r="C19" s="7">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C20" s="7">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>1277</v>
+      </c>
+      <c r="C21" s="7">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>1278</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C22" s="7">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C23" s="7">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C24" s="7">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>1284</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C25" s="7">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C26" s="7">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C27" s="7">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C28" s="7">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>1292</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C29" s="7">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C30" s="7">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C31" s="7">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>1299</v>
+      </c>
+      <c r="C32" s="7">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C33" s="7">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C34" s="7">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>1305</v>
+      </c>
+      <c r="C35" s="7">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C36" s="7">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C37" s="7"/>
+    </row>
+    <row r="38" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>1311</v>
+      </c>
+      <c r="C38" s="7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C39" s="7">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C40" s="7">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C41" s="7">
+        <v>2326</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C42" s="7">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C43" s="7">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C44" s="7">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C45" s="7">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="C46" s="7">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="C47" s="7">
+        <v>2168</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C48" s="7">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>1332</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C49" s="7">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>1335</v>
+      </c>
+      <c r="C50" s="7">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>1337</v>
+      </c>
+      <c r="C51" s="7">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C52" s="7">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C53" s="7">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C54" s="7">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
+        <v>1344</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>1345</v>
+      </c>
+      <c r="C55" s="7">
+        <v>1252</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="6" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>1347</v>
+      </c>
+      <c r="C56" s="7">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
+        <v>1348</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C57" s="7">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>1351</v>
+      </c>
+      <c r="C58" s="7">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
+        <v>1352</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C59" s="7">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C60" s="7">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
+        <v>1356</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C61" s="7">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C62" s="7">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
+        <v>1360</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C63" s="7">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="6" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>1363</v>
+      </c>
+      <c r="C64" s="7">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
+        <v>1364</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C65" s="7">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="6" t="s">
+        <v>1366</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C66" s="7">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
+        <v>1368</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C67" s="7">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="6" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C68" s="7">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C69" s="7">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="6" t="s">
+        <v>1374</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C70" s="7">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C71" s="7">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="6" t="s">
+        <v>1378</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C72" s="7">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="6" t="s">
+        <v>1380</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C73" s="7">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>1382</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>1383</v>
+      </c>
+      <c r="C74" s="7">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="6" t="s">
+        <v>1384</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C75" s="7">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="6" t="s">
+        <v>1386</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C76" s="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="6" t="s">
+        <v>1388</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C77" s="7">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="6" t="s">
+        <v>1390</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C78" s="7">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="6" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C79" s="7">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>1394</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C80" s="7">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="6" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C81" s="7">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>1399</v>
+      </c>
+      <c r="C82" s="7">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="6" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C83" s="7"/>
+    </row>
+    <row r="84" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="6" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C84" s="7">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="6" t="s">
+        <v>1404</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C85" s="7">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>1406</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C86" s="7">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="6" t="s">
+        <v>1408</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>1409</v>
+      </c>
+      <c r="C87" s="7">
+        <v>1511</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="6" t="s">
+        <v>1410</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>1411</v>
+      </c>
+      <c r="C88" s="7">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="6" t="s">
+        <v>1412</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>1413</v>
+      </c>
+      <c r="C89" s="7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
+        <v>1414</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>1415</v>
+      </c>
+      <c r="C90" s="7">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="6" t="s">
+        <v>1416</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>1417</v>
+      </c>
+      <c r="C91" s="7">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>1418</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>1419</v>
+      </c>
+      <c r="C92" s="7">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="6" t="s">
+        <v>1420</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C93" s="7">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="6" t="s">
+        <v>1422</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C94" s="7">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="6" t="s">
+        <v>1424</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>1425</v>
+      </c>
+      <c r="C95" s="7">
+        <v>2315</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="6" t="s">
+        <v>1426</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C96" s="7">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="6" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C97" s="7">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="6" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C98" s="7">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="6" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C99" s="7">
+        <v>2377</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="6" t="s">
+        <v>1434</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C100" s="7">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="6" t="s">
+        <v>1436</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C101" s="7">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="6" t="s">
+        <v>1438</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>1439</v>
+      </c>
+      <c r="C102" s="7">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="6" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C103" s="7">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="6" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C104" s="7">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="6" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C105" s="7">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="6" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>1447</v>
+      </c>
+      <c r="C106" s="7">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="6" t="s">
+        <v>1448</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>1449</v>
+      </c>
+      <c r="C107" s="7">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="6" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C108" s="7">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="6" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>1453</v>
+      </c>
+      <c r="C109" s="7">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="6" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C110" s="7">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="6" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C111" s="7">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="6" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C112" s="7">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="6" t="s">
+        <v>1460</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>1461</v>
+      </c>
+      <c r="C113" s="7">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="6" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>1463</v>
+      </c>
+      <c r="C114" s="7">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="6" t="s">
+        <v>1464</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C115" s="7">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="6" t="s">
+        <v>1466</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>1467</v>
+      </c>
+      <c r="C116" s="7">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="6" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>1469</v>
+      </c>
+      <c r="C117" s="7">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="6" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C118" s="7">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="6" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C119" s="7">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="6" t="s">
+        <v>1474</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>1475</v>
+      </c>
+      <c r="C120" s="7">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="6" t="s">
+        <v>1476</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C121" s="7">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="6" t="s">
+        <v>1478</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>1479</v>
+      </c>
+      <c r="C122" s="7">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="6" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>1481</v>
+      </c>
+      <c r="C123" s="7">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="6" t="s">
+        <v>1482</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C124" s="7">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="6" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C125" s="7">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="6" t="s">
+        <v>1486</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C126" s="7"/>
+    </row>
+    <row r="127" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="6" t="s">
+        <v>1488</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>1489</v>
+      </c>
+      <c r="C127" s="7">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="6" t="s">
+        <v>1490</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C128" s="7">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="6" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C129" s="7">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="6" t="s">
+        <v>1494</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C130" s="7">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="6" t="s">
+        <v>1496</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C131" s="7">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="6" t="s">
+        <v>1498</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C132" s="7">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="6" t="s">
+        <v>1500</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C133" s="7">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="6" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C134" s="7">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="6" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>1505</v>
+      </c>
+      <c r="C135" s="7">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="6" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C136" s="7">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="6" t="s">
+        <v>1508</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>1509</v>
+      </c>
+      <c r="C137" s="7">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="6" t="s">
+        <v>1510</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C138" s="7">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="6" t="s">
+        <v>1512</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C139" s="7">
+        <v>2411</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="6" t="s">
+        <v>1514</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>1515</v>
+      </c>
+      <c r="C140" s="7">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="6" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>1517</v>
+      </c>
+      <c r="C141" s="7">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="6" t="s">
+        <v>1518</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C142" s="7"/>
+    </row>
+    <row r="143" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="6" t="s">
+        <v>1520</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>1521</v>
+      </c>
+      <c r="C143" s="7">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A144" s="6" t="s">
+        <v>1522</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>1523</v>
+      </c>
+      <c r="C144" s="7">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>1524</v>
+      </c>
+      <c r="C145" s="7">
+        <v>1761</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="6" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>1526</v>
+      </c>
+      <c r="C146" s="7">
+        <v>1409</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="6" t="s">
+        <v>1527</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C147" s="7">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="6" t="s">
+        <v>1529</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C148" s="7">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="6" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>1532</v>
+      </c>
+      <c r="C149" s="7">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="6" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C150" s="7"/>
+    </row>
+    <row r="151" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="6" t="s">
+        <v>1535</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>1536</v>
+      </c>
+      <c r="C151" s="7">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="6" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>1538</v>
+      </c>
+      <c r="C152" s="7">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>1551</v>
+      </c>
+      <c r="C153" s="7"/>
+    </row>
+    <row r="154" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A154" s="6" t="s">
+        <v>1540</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>1541</v>
+      </c>
+      <c r="C154" s="7">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="6" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>1543</v>
+      </c>
+      <c r="C155" s="7"/>
+    </row>
+    <row r="156" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="6" t="s">
+        <v>1544</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>1545</v>
+      </c>
+      <c r="C156" s="7"/>
+    </row>
+    <row r="157" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="6" t="s">
+        <v>1546</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C157" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Move subsection/classification code lookup to the main lookup .xlsx file
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tpoongundranar\Documents\Urban\NCCS\nccs-data-bmf\data\lookup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6569F1-4400-4902-AD61-11DF37067A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D53A0F3-E5E7-493F-BFE0-18DC2F79B7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="9" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
   </bookViews>
   <sheets>
     <sheet name="status_code" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="ntee_code_activity_type" sheetId="7" r:id="rId7"/>
     <sheet name="ntee_code_major_group" sheetId="8" r:id="rId8"/>
     <sheet name="parent_organization" sheetId="9" r:id="rId9"/>
+    <sheet name="subsection_classification_code" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="1552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="1656">
   <si>
     <t>status_code</t>
   </si>
@@ -4700,6 +4701,318 @@
   </si>
   <si>
     <t>PTA</t>
+  </si>
+  <si>
+    <t>subsection_code</t>
+  </si>
+  <si>
+    <t>classification_code</t>
+  </si>
+  <si>
+    <t>classification_description</t>
+  </si>
+  <si>
+    <t>exempt_organization_type</t>
+  </si>
+  <si>
+    <t>effective_start_date</t>
+  </si>
+  <si>
+    <t>effective_end_date</t>
+  </si>
+  <si>
+    <t>Government instrumentality</t>
+  </si>
+  <si>
+    <t>501(c)(1)</t>
+  </si>
+  <si>
+    <t>Title-holding corporation</t>
+  </si>
+  <si>
+    <t>501(c)(2)</t>
+  </si>
+  <si>
+    <t>Charitable Organization</t>
+  </si>
+  <si>
+    <t>501(c)(3)</t>
+  </si>
+  <si>
+    <t>Educational organization</t>
+  </si>
+  <si>
+    <t>Literary organization</t>
+  </si>
+  <si>
+    <t>Organization to prevent cruelty to animals</t>
+  </si>
+  <si>
+    <t>Organization to prevent cruelty to children</t>
+  </si>
+  <si>
+    <t>Organization for public safety testing</t>
+  </si>
+  <si>
+    <t>Religious organization</t>
+  </si>
+  <si>
+    <t>Scientific organization</t>
+  </si>
+  <si>
+    <t>Civic league</t>
+  </si>
+  <si>
+    <t>501(c)(4)</t>
+  </si>
+  <si>
+    <t>Local association of employees</t>
+  </si>
+  <si>
+    <t>Social welfare organization</t>
+  </si>
+  <si>
+    <t>Agriculture organization</t>
+  </si>
+  <si>
+    <t>501(c)(5)</t>
+  </si>
+  <si>
+    <t>Horticulture organization</t>
+  </si>
+  <si>
+    <t>Labor organization</t>
+  </si>
+  <si>
+    <t>Board of Trade</t>
+  </si>
+  <si>
+    <t>501(c)(6)</t>
+  </si>
+  <si>
+    <t>Business league</t>
+  </si>
+  <si>
+    <t>Chamber of Commerce</t>
+  </si>
+  <si>
+    <t>Real estate board</t>
+  </si>
+  <si>
+    <t>Pleasure, recreational, or social club</t>
+  </si>
+  <si>
+    <t>501(c)(7)</t>
+  </si>
+  <si>
+    <t>Fraternal beneficiary society, order or association</t>
+  </si>
+  <si>
+    <t>501(c)(8)</t>
+  </si>
+  <si>
+    <t>Voluntary employees’ beneficiary association (Non-government)</t>
+  </si>
+  <si>
+    <t>501(c)(9)</t>
+  </si>
+  <si>
+    <t>Voluntary employees’ beneficiary association (Government emp.’s)</t>
+  </si>
+  <si>
+    <t>Domestic fraternal societies and associations</t>
+  </si>
+  <si>
+    <t>501(c)(10)</t>
+  </si>
+  <si>
+    <t>Teachers’ retirement fund association</t>
+  </si>
+  <si>
+    <t>501(c)(11)</t>
+  </si>
+  <si>
+    <t>Benevolent life insurance association</t>
+  </si>
+  <si>
+    <t>501(c)(12)</t>
+  </si>
+  <si>
+    <t>Mutual ditch or irrigation company</t>
+  </si>
+  <si>
+    <t>Mutual or cooperative telephone company</t>
+  </si>
+  <si>
+    <t>Mutual electric company, mutual water company, etc.</t>
+  </si>
+  <si>
+    <t>Burial association</t>
+  </si>
+  <si>
+    <t>501(c)(13)</t>
+  </si>
+  <si>
+    <t>Cemetery company</t>
+  </si>
+  <si>
+    <t>Credit Union</t>
+  </si>
+  <si>
+    <t>501(c)(14)</t>
+  </si>
+  <si>
+    <t>Other mutual corporation or association</t>
+  </si>
+  <si>
+    <t>Mutual insurance company or association other than life or marine</t>
+  </si>
+  <si>
+    <t>501(c)(15)</t>
+  </si>
+  <si>
+    <t>Corporation financing crop operation</t>
+  </si>
+  <si>
+    <t>501(c)(16)</t>
+  </si>
+  <si>
+    <t>Supplemental unemployment compensation trust or plan</t>
+  </si>
+  <si>
+    <t>501(c)(17)</t>
+  </si>
+  <si>
+    <t>Employee funded pension trust (created before 6–25–59)</t>
+  </si>
+  <si>
+    <t>501(c)(18)</t>
+  </si>
+  <si>
+    <t>Post or organization of war veterans</t>
+  </si>
+  <si>
+    <t>501(c)(19)</t>
+  </si>
+  <si>
+    <t>Legal Services Organization</t>
+  </si>
+  <si>
+    <t>501(c)(20)</t>
+  </si>
+  <si>
+    <t>Black Lung</t>
+  </si>
+  <si>
+    <t>501(c)(21)</t>
+  </si>
+  <si>
+    <t>Multiemployer Pension Plan</t>
+  </si>
+  <si>
+    <t>501(c)(22)</t>
+  </si>
+  <si>
+    <t>Veterans Association Founded Prior to 1880</t>
+  </si>
+  <si>
+    <t>501(c)(23)</t>
+  </si>
+  <si>
+    <t>Trust described in Section 4049 of ERISA</t>
+  </si>
+  <si>
+    <t>501(c)(24)</t>
+  </si>
+  <si>
+    <t>Title Holding Corporation or Trust</t>
+  </si>
+  <si>
+    <t>501(c)(25)</t>
+  </si>
+  <si>
+    <t>State-sponsored High-Risk Health Insurance Org. Effective (1/1/99)</t>
+  </si>
+  <si>
+    <t>501(c)(26)</t>
+  </si>
+  <si>
+    <t>State-sponsored Worker’s Compensation Reinsurance Organization (Effective 1/1/99)</t>
+  </si>
+  <si>
+    <t>501(c)(27)</t>
+  </si>
+  <si>
+    <t>National Railroad Retirement Investment Trust Classification</t>
+  </si>
+  <si>
+    <t>501(c)(28)</t>
+  </si>
+  <si>
+    <t>Qualified non profit Health Insurance Issuers</t>
+  </si>
+  <si>
+    <t>501(c)(29)</t>
+  </si>
+  <si>
+    <t>Apostolic and religious organization</t>
+  </si>
+  <si>
+    <t>501(d)</t>
+  </si>
+  <si>
+    <t>Cooperative hospital service organization</t>
+  </si>
+  <si>
+    <t>501(e)</t>
+  </si>
+  <si>
+    <t>Cooperative service organizations of operating education org’s</t>
+  </si>
+  <si>
+    <t>501(f)</t>
+  </si>
+  <si>
+    <t>Child care under 501(k)</t>
+  </si>
+  <si>
+    <t>501(k)</t>
+  </si>
+  <si>
+    <t>Charitable Risk Pool (Effective 1/1/99)</t>
+  </si>
+  <si>
+    <t>501(n)</t>
+  </si>
+  <si>
+    <t>Farmers’ Cooperative</t>
+  </si>
+  <si>
+    <t>Qualified State-Sponsored Tuition Program</t>
+  </si>
+  <si>
+    <t>IRC 527</t>
+  </si>
+  <si>
+    <t>Non-exempt charitable trust 4947(a)(2) (Split Interest)</t>
+  </si>
+  <si>
+    <t>4947(a)(2)</t>
+  </si>
+  <si>
+    <t>Non-exempt charitable trust (Public Charity)</t>
+  </si>
+  <si>
+    <t>4947(a)(1)</t>
+  </si>
+  <si>
+    <t>Non-exempt charitable trust (Trust treated as Private Foundation)</t>
+  </si>
+  <si>
+    <t>Taxable Farmer’s Cooperative</t>
+  </si>
+  <si>
+    <t>1381(a)(2)</t>
   </si>
 </sst>
 </file>
@@ -5199,6 +5512,1256 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B298717-5B0C-43D8-96E1-9B90896F2A43}">
+  <dimension ref="A1:F62"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1552</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1553</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1554</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1555</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1556</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1558</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1559</v>
+      </c>
+      <c r="E2">
+        <v>20241213</v>
+      </c>
+      <c r="F2">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1560</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1561</v>
+      </c>
+      <c r="E3">
+        <v>20241213</v>
+      </c>
+      <c r="F3">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E4">
+        <v>20241213</v>
+      </c>
+      <c r="F4">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1564</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E5">
+        <v>20241213</v>
+      </c>
+      <c r="F5">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1565</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E6">
+        <v>20241213</v>
+      </c>
+      <c r="F6">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1566</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E7">
+        <v>20241213</v>
+      </c>
+      <c r="F7">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E8">
+        <v>20241213</v>
+      </c>
+      <c r="F8">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1568</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E9">
+        <v>20241213</v>
+      </c>
+      <c r="F9">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1569</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E10">
+        <v>20241213</v>
+      </c>
+      <c r="F10">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1570</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E11">
+        <v>20241213</v>
+      </c>
+      <c r="F11">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1571</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1572</v>
+      </c>
+      <c r="E12">
+        <v>20241213</v>
+      </c>
+      <c r="F12">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1573</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1572</v>
+      </c>
+      <c r="E13">
+        <v>20241213</v>
+      </c>
+      <c r="F13">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>4</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1574</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1572</v>
+      </c>
+      <c r="E14">
+        <v>20241213</v>
+      </c>
+      <c r="F14">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1575</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1576</v>
+      </c>
+      <c r="E15">
+        <v>20241213</v>
+      </c>
+      <c r="F15">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1577</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1576</v>
+      </c>
+      <c r="E16">
+        <v>20241213</v>
+      </c>
+      <c r="F16">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>5</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1578</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1576</v>
+      </c>
+      <c r="E17">
+        <v>20241213</v>
+      </c>
+      <c r="F17">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1579</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1580</v>
+      </c>
+      <c r="E18">
+        <v>20241213</v>
+      </c>
+      <c r="F18">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1581</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1580</v>
+      </c>
+      <c r="E19">
+        <v>20241213</v>
+      </c>
+      <c r="F19">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>6</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1582</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1580</v>
+      </c>
+      <c r="E20">
+        <v>20241213</v>
+      </c>
+      <c r="F20">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>6</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1583</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1580</v>
+      </c>
+      <c r="E21">
+        <v>20241213</v>
+      </c>
+      <c r="F21">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>7</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1584</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1585</v>
+      </c>
+      <c r="E22">
+        <v>20241213</v>
+      </c>
+      <c r="F22">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>8</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1586</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1587</v>
+      </c>
+      <c r="E23">
+        <v>20241213</v>
+      </c>
+      <c r="F23">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>9</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1588</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1589</v>
+      </c>
+      <c r="E24">
+        <v>20241213</v>
+      </c>
+      <c r="F24">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>9</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1590</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1589</v>
+      </c>
+      <c r="E25">
+        <v>20241213</v>
+      </c>
+      <c r="F25">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>10</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1591</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1592</v>
+      </c>
+      <c r="E26">
+        <v>20241213</v>
+      </c>
+      <c r="F26">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>11</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1593</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1594</v>
+      </c>
+      <c r="E27">
+        <v>20241213</v>
+      </c>
+      <c r="F27">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>12</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1595</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1596</v>
+      </c>
+      <c r="E28">
+        <v>20241213</v>
+      </c>
+      <c r="F28">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>12</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1597</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1596</v>
+      </c>
+      <c r="E29">
+        <v>20241213</v>
+      </c>
+      <c r="F29">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>12</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1598</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1596</v>
+      </c>
+      <c r="E30">
+        <v>20241213</v>
+      </c>
+      <c r="F30">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>12</v>
+      </c>
+      <c r="B31">
+        <v>4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1599</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1596</v>
+      </c>
+      <c r="E31">
+        <v>20241213</v>
+      </c>
+      <c r="F31">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>13</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1600</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1601</v>
+      </c>
+      <c r="E32">
+        <v>20241213</v>
+      </c>
+      <c r="F32">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>13</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1602</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1601</v>
+      </c>
+      <c r="E33">
+        <v>20241213</v>
+      </c>
+      <c r="F33">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>14</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E34">
+        <v>20241213</v>
+      </c>
+      <c r="F34">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>14</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1605</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E35">
+        <v>20241213</v>
+      </c>
+      <c r="F35">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>15</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1606</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1607</v>
+      </c>
+      <c r="E36">
+        <v>20241213</v>
+      </c>
+      <c r="F36">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>16</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1608</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1609</v>
+      </c>
+      <c r="E37">
+        <v>20241213</v>
+      </c>
+      <c r="F37">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>17</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1610</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1611</v>
+      </c>
+      <c r="E38">
+        <v>20241213</v>
+      </c>
+      <c r="F38">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>18</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1612</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1613</v>
+      </c>
+      <c r="E39">
+        <v>20241213</v>
+      </c>
+      <c r="F39">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>19</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1614</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1615</v>
+      </c>
+      <c r="E40">
+        <v>20241213</v>
+      </c>
+      <c r="F40">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>20</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1616</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1617</v>
+      </c>
+      <c r="E41">
+        <v>20241213</v>
+      </c>
+      <c r="F41">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>21</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1618</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1619</v>
+      </c>
+      <c r="E42">
+        <v>20241213</v>
+      </c>
+      <c r="F42">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>22</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1620</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1621</v>
+      </c>
+      <c r="E43">
+        <v>20241213</v>
+      </c>
+      <c r="F43">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>23</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1622</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1623</v>
+      </c>
+      <c r="E44">
+        <v>20241213</v>
+      </c>
+      <c r="F44">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>24</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1625</v>
+      </c>
+      <c r="E45">
+        <v>20241213</v>
+      </c>
+      <c r="F45">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>25</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1627</v>
+      </c>
+      <c r="E46">
+        <v>20241213</v>
+      </c>
+      <c r="F46">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>26</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1628</v>
+      </c>
+      <c r="D47" t="s">
+        <v>1629</v>
+      </c>
+      <c r="E47">
+        <v>20241213</v>
+      </c>
+      <c r="F47">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>27</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D48" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E48">
+        <v>20241213</v>
+      </c>
+      <c r="F48">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>28</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1632</v>
+      </c>
+      <c r="D49" t="s">
+        <v>1633</v>
+      </c>
+      <c r="E49">
+        <v>20241213</v>
+      </c>
+      <c r="F49">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>29</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D50" t="s">
+        <v>1635</v>
+      </c>
+      <c r="E50">
+        <v>20241213</v>
+      </c>
+      <c r="F50">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>40</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1636</v>
+      </c>
+      <c r="D51" t="s">
+        <v>1637</v>
+      </c>
+      <c r="E51">
+        <v>20241213</v>
+      </c>
+      <c r="F51">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>50</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D52" t="s">
+        <v>1639</v>
+      </c>
+      <c r="E52">
+        <v>20241213</v>
+      </c>
+      <c r="F52">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>60</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1640</v>
+      </c>
+      <c r="D53" t="s">
+        <v>1641</v>
+      </c>
+      <c r="E53">
+        <v>20241213</v>
+      </c>
+      <c r="F53">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>70</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1642</v>
+      </c>
+      <c r="D54" t="s">
+        <v>1643</v>
+      </c>
+      <c r="E54">
+        <v>20241213</v>
+      </c>
+      <c r="F54">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>71</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1644</v>
+      </c>
+      <c r="D55" t="s">
+        <v>1645</v>
+      </c>
+      <c r="E55">
+        <v>20241213</v>
+      </c>
+      <c r="F55">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>80</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1646</v>
+      </c>
+      <c r="D56">
+        <v>521</v>
+      </c>
+      <c r="E56">
+        <v>20241213</v>
+      </c>
+      <c r="F56">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>81</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1647</v>
+      </c>
+      <c r="D57">
+        <v>529</v>
+      </c>
+      <c r="E57">
+        <v>20241213</v>
+      </c>
+      <c r="F57">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>82</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1648</v>
+      </c>
+      <c r="D58">
+        <v>82</v>
+      </c>
+      <c r="E58">
+        <v>20241213</v>
+      </c>
+      <c r="F58">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>90</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1649</v>
+      </c>
+      <c r="D59" t="s">
+        <v>1650</v>
+      </c>
+      <c r="E59">
+        <v>20241213</v>
+      </c>
+      <c r="F59">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>91</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1651</v>
+      </c>
+      <c r="D60" t="s">
+        <v>1652</v>
+      </c>
+      <c r="E60">
+        <v>20241213</v>
+      </c>
+      <c r="F60">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>92</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1653</v>
+      </c>
+      <c r="D61" t="s">
+        <v>1652</v>
+      </c>
+      <c r="E61">
+        <v>20241213</v>
+      </c>
+      <c r="F61">
+        <v>99991231</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>93</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
+        <v>1654</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1655</v>
+      </c>
+      <c r="E62">
+        <v>20241213</v>
+      </c>
+      <c r="F62">
+        <v>99991231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28F26964-D323-4807-93C3-4339F47CA786}">
   <dimension ref="A1:C11"/>

</xml_diff>

<commit_message>
Move affiliation code lookup to main lookup file
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tpoongundranar\Documents\Urban\NCCS\nccs-data-bmf\data\lookup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D53A0F3-E5E7-493F-BFE0-18DC2F79B7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E71EF2-EBC7-4F5E-A034-7453DB528E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="9" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="10" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
   </bookViews>
   <sheets>
     <sheet name="status_code" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="ntee_code_major_group" sheetId="8" r:id="rId8"/>
     <sheet name="parent_organization" sheetId="9" r:id="rId9"/>
     <sheet name="subsection_classification_code" sheetId="10" r:id="rId10"/>
+    <sheet name="affiliation_code" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="1656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1891" uniqueCount="1673">
   <si>
     <t>status_code</t>
   </si>
@@ -5013,6 +5014,63 @@
   </si>
   <si>
     <t>1381(a)(2)</t>
+  </si>
+  <si>
+    <t>affiliation_code</t>
+  </si>
+  <si>
+    <t>affiliation_code_definition</t>
+  </si>
+  <si>
+    <t>affiliation_code_description</t>
+  </si>
+  <si>
+    <t>Central Organization (Individual Ruling)</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is a central type organization (no group exemption) of a National,_x000D_
+Regional or Geographic grouping of organizations.</t>
+  </si>
+  <si>
+    <t>Intermediate Organization (Individual Ruling)</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is an intermediate organization (no group exemption) of a_x000D_
+National, Regional or Geographic grouping of organizations (such as a state headquarters of a national_x000D_
+organization).</t>
+  </si>
+  <si>
+    <t>Independent organization (Individual Ruling)</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is an independent organization or an independent auxiliary_x000D_
+(i.e., not affiliated with a National, Regional, or Geographic grouping of organizations).</t>
+  </si>
+  <si>
+    <t>Parent of a group ruling (not a church)</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is a parent (group ruling) and is not a church or 501(c)(1)_x000D_
+organization.</t>
+  </si>
+  <si>
+    <t>Intermediate parent (subordinate by state)</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is a group exemption intermediate organization of a National,_x000D_
+Regional or Geographic grouping of organizations.</t>
+  </si>
+  <si>
+    <t>Parent of a church</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is a parent (group ruling) and is a church or 501(c)(1) organization.</t>
+  </si>
+  <si>
+    <t>Subordinate of a group ruling (also, group return)</t>
+  </si>
+  <si>
+    <t>This code is used if the organization is a subordinate in a group ruling.</t>
   </si>
 </sst>
 </file>
@@ -6762,6 +6820,104 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B295775B-C545-42EF-B1E6-C8444CDB5163}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1656</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1657</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1658</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1659</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1663</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1664</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1665</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1666</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1667</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1668</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1669</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1671</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1672</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28F26964-D323-4807-93C3-4339F47CA786}">
   <dimension ref="A1:C11"/>

</xml_diff>

<commit_message>
Move deductibility code lookup into main lookup
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tpoongundranar\Documents\Urban\NCCS\nccs-data-bmf\data\lookup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E71EF2-EBC7-4F5E-A034-7453DB528E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC1D010-B9D6-4E7E-9E65-567729AE50E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="10" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="11" xr2:uid="{1B4F8980-FB82-4AA6-95DF-3A9E10ACA6D4}"/>
   </bookViews>
   <sheets>
     <sheet name="status_code" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="parent_organization" sheetId="9" r:id="rId9"/>
     <sheet name="subsection_classification_code" sheetId="10" r:id="rId10"/>
     <sheet name="affiliation_code" sheetId="11" r:id="rId11"/>
+    <sheet name="deductibility_code" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1891" uniqueCount="1673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1899" uniqueCount="1681">
   <si>
     <t>status_code</t>
   </si>
@@ -5071,6 +5072,30 @@
   </si>
   <si>
     <t>This code is used if the organization is a subordinate in a group ruling.</t>
+  </si>
+  <si>
+    <t>deductibility_code</t>
+  </si>
+  <si>
+    <t>deductibility_code_definition</t>
+  </si>
+  <si>
+    <t>deductibility_code_start_date</t>
+  </si>
+  <si>
+    <t>deductibility_code_end_date</t>
+  </si>
+  <si>
+    <t>Contributions are deductible</t>
+  </si>
+  <si>
+    <t>Contributions aren't deductible</t>
+  </si>
+  <si>
+    <t>Contributions are deductible under treaty provisions</t>
+  </si>
+  <si>
+    <t>Undefined</t>
   </si>
 </sst>
 </file>
@@ -6918,6 +6943,74 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A251961A-4424-404F-8F77-6EB707D782F5}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1673</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1674</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1675</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1676</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1677</v>
+      </c>
+      <c r="C2">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1678</v>
+      </c>
+      <c r="C3">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1679</v>
+      </c>
+      <c r="C4">
+        <v>20241213</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C5">
+        <v>20241213</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28F26964-D323-4807-93C3-4339F47CA786}">
   <dimension ref="A1:C11"/>

</xml_diff>